<commit_message>
数据更新 8/12 MD-3 50min
</commit_message>
<xml_diff>
--- a/public/share/data/每日强度监控.xlsx
+++ b/public/share/data/每日强度监控.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24460" windowHeight="11120" tabRatio="600" firstSheet="29" activeTab="33" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24460" windowHeight="11120" tabRatio="600" firstSheet="29" activeTab="34" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7.06" sheetId="1" state="visible" r:id="rId1"/>
@@ -40,6 +40,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8.8" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8.9" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8.11" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8.12" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -28666,8 +28667,6 @@
       <c r="H4" t="n">
         <v>120</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -28698,25 +28697,966 @@
       <c r="H5" t="n">
         <v>180</v>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>努尔扎提-努尔兰</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>60</v>
+      </c>
+      <c r="H6" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>吕佳骏</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>60</v>
+      </c>
+      <c r="H7" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>巫林峰</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H8" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>布格拉汗-斯坎旦尔</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>60</v>
+      </c>
+      <c r="H9" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>帕尔曼江-克尤木</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>60</v>
+      </c>
+      <c r="H10" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>张俊哲</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>60</v>
+      </c>
+      <c r="H11" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>张天龙</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
+        <v>60</v>
+      </c>
+      <c r="H12" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>张海轩</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>60</v>
+      </c>
+      <c r="H13" t="n">
+        <v>180</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>脚踝痛D6</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>继续冰敷+踝泵</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>张辉</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="n">
+        <v>60</v>
+      </c>
+      <c r="H14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>脚腕微痛🆕</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>朱云天(U21)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>60</v>
+      </c>
+      <c r="H15" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>杨卓燠</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>60</v>
+      </c>
+      <c r="H16" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>杨文杰</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>60</v>
+      </c>
+      <c r="H17" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>杨翼璇</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="n">
+        <v>60</v>
+      </c>
+      <c r="H18" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>林楷轩(U21)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" t="n">
+        <v>60</v>
+      </c>
+      <c r="H19" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>栾昊(U21)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" t="n">
+        <v>60</v>
+      </c>
+      <c r="H20" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>王捷(U21)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" t="n">
+        <v>60</v>
+      </c>
+      <c r="H21" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>王款(U21)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
+        <v>60</v>
+      </c>
+      <c r="H22" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>王熙博</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" t="n">
+        <v>60</v>
+      </c>
+      <c r="H23" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>王皓文(U21)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" t="n">
+        <v>60</v>
+      </c>
+      <c r="H24" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>艾沙江-库尔班</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>60</v>
+      </c>
+      <c r="H25" t="n">
+        <v>300</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>RPE=5·赛前MCL疼</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>D+3降负荷·避免冲刺</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>阿西江-白山</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" t="n">
+        <v>60</v>
+      </c>
+      <c r="H26" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>陈少豪</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="n">
+        <v>60</v>
+      </c>
+      <c r="H27" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>陈祥煜</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" t="n">
+        <v>60</v>
+      </c>
+      <c r="H28" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>谢锦政</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>李金羽</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>董德</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>训练50min</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>球员</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>位置</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RPE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>睡眠</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>疲劳</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>酸痛</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>时长</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>sRPE</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>建议</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>张海轩</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>门将</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>脚踝疼持续5天</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>持续观察，赛前评估</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>杨卓燠</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>门将</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H5" t="n">
+        <v>150</v>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>努尔扎提-努尔兰</t>
+          <t>王款(U21)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>门将</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -28725,10 +29665,10 @@
         <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H6" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -28736,12 +29676,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>吕佳骏</t>
+          <t>王熙博</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>门将</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -28757,10 +29697,10 @@
         <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H7" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -28768,31 +29708,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>巫林峰</t>
+          <t>张俊哲</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H8" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -28800,16 +29740,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>布格拉汗-斯坎旦尔</t>
+          <t>张天龙</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -28821,10 +29761,10 @@
         <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H9" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -28832,31 +29772,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>帕尔曼江-克尤木</t>
+          <t>凌中阳</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H10" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -28864,12 +29804,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>张俊哲</t>
+          <t>陈少豪</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -28879,16 +29819,16 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H11" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -28896,16 +29836,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>张天龙</t>
+          <t>李金羽</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
@@ -28917,10 +29857,10 @@
         <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H12" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -28928,12 +29868,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>张海轩</t>
+          <t>王捷(U21)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -28943,128 +29883,136 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H13" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>脚踝痛D6</t>
+          <t>左膝髌腱炎持续</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>继续冰敷+踝泵</t>
+          <t>控制跳跃急停负荷</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>张辉</t>
+          <t>王皓文(U21)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
         <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H14" t="n">
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>脚腕微痛🆕</t>
+          <t>RPE偏高</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>观察</t>
+          <t>MD-3窗口内可接受</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>朱云天(U21)</t>
+          <t>丁云峰</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H15" t="n">
-        <v>180</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+        <v>150</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>睡眠4偏高</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>关注恢复</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>杨卓燠</t>
+          <t>杨文杰</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>后卫</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H16" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -29072,51 +30020,45 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>杨文杰</t>
+          <t>刘子洁</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
+          <t>后卫</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="n">
         <v>2</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" t="n">
-        <v>60</v>
-      </c>
-      <c r="H17" t="n">
-        <v>180</v>
-      </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>未参训</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>杨翼璇</t>
+          <t>何麟立</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
@@ -29125,30 +30067,38 @@
         <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H18" t="n">
-        <v>120</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+        <v>250</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>内收肌还是有点紧</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>持续关注，MD-2减量</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>林楷轩(U21)</t>
+          <t>布格拉汗-斯坎旦尔</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
@@ -29157,10 +30107,10 @@
         <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H19" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -29168,19 +30118,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>栾昊(U21)</t>
+          <t>巫林峰</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
@@ -29189,10 +30139,10 @@
         <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H20" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -29200,49 +30150,55 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>王捷(U21)</t>
+          <t>张辉</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G21" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H21" t="n">
-        <v>180</v>
-      </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+        <v>300</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>本周最高RPE</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>MD-3峰值可接受</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>王款(U21)</t>
+          <t>谢锦政</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GK</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
+          <t>中场</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="n">
         <v>2</v>
       </c>
@@ -29252,31 +30208,35 @@
       <c r="F22" t="n">
         <v>2</v>
       </c>
-      <c r="G22" t="n">
-        <v>60</v>
-      </c>
-      <c r="H22" t="n">
-        <v>120</v>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>脚趾恢复中，未参训</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>继续观察</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>王熙博</t>
+          <t>栾昊(U21)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
         <v>2</v>
@@ -29285,10 +30245,10 @@
         <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H23" t="n">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -29296,31 +30256,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>王皓文(U21)</t>
+          <t>杨翼璇</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G24" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H24" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -29328,116 +30288,108 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>艾沙江-库尔班</t>
+          <t>林楷轩(U21)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
         <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H25" t="n">
-        <v>300</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>RPE=5·赛前MCL疼</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>D+3降负荷·避免冲刺</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>阿西江-白山</t>
+          <t>朱云天(U21)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H26" t="n">
-        <v>180</v>
-      </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+        <v>300</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>本周最高RPE</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>MD-3峰值可接受</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>陈少豪</t>
+          <t>董德</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" t="n">
-        <v>60</v>
-      </c>
-      <c r="H27" t="n">
-        <v>120</v>
-      </c>
-      <c r="I27" t="inlineStr"/>
+          <t>中场</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>未参训</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>陈祥煜</t>
+          <t>吕佳骏</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>中场</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -29453,10 +30405,10 @@
         <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H28" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -29464,15 +30416,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>谢锦政</t>
+          <t>陈祥煜</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>前锋</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
       <c r="D29" t="n">
         <v>2</v>
       </c>
@@ -29480,64 +30434,152 @@
         <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>50</v>
+      </c>
+      <c r="H29" t="n">
+        <v>150</v>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>李金羽</t>
+          <t>艾沙江-库尔班</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>前锋</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>5</v>
+      </c>
       <c r="D30" t="n">
         <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G30" t="n">
+        <v>50</v>
+      </c>
+      <c r="H30" t="n">
+        <v>250</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>疲劳酸痛偏高</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>MCL史，关注</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>董德</t>
+          <t>帕尔曼江-克尤木</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>前锋</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G31" t="n">
+        <v>50</v>
+      </c>
+      <c r="H31" t="n">
+        <v>200</v>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>阿西江-白山</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>前锋</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" t="n">
+        <v>50</v>
+      </c>
+      <c r="H32" t="n">
+        <v>200</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>努尔扎提-努尔兰</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>前锋</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" t="n">
+        <v>50</v>
+      </c>
+      <c r="H33" t="n">
+        <v>200</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>